<commit_message>
test: verify forced question progression
</commit_message>
<xml_diff>
--- a/content/generated/script.generated.xlsx
+++ b/content/generated/script.generated.xlsx
@@ -23,7 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterTable" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterEmotionTable" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuestionTable" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StateDescriptorTable" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuestionAnswerTable" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StateDescriptorTable" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-12 21:04:29</t>
+          <t>2026-08-12 22:51:25</t>
         </is>
       </c>
     </row>
@@ -488,7 +489,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ConditionTable, GaugeTable, GaugeStateTable, EffectTable, SceneTable, DialogTable, ChoiceGroupTable, ChoiceTable, BranchTable, EvidenceTable, EvidenceCategoryTable, CharacterTable, CharacterEmotionTable, QuestionTable, StateDescriptorTable</t>
+          <t>ConditionTable, GaugeTable, GaugeStateTable, EffectTable, SceneTable, DialogTable, ChoiceGroupTable, ChoiceTable, BranchTable, EvidenceTable, EvidenceCategoryTable, CharacterTable, CharacterEmotionTable, QuestionTable, QuestionAnswerTable, StateDescriptorTable</t>
         </is>
       </c>
     </row>
@@ -599,7 +600,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>이 판결, 기어이 물고 늘어진다.</t>
+          <t>판결문에서 푸른 천과 이판규의 시선을 따로 기록한다.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -629,7 +630,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>편집장이 원하는 기사를 먼저 써둔다. 그게 실리는 법이다.</t>
+          <t>판결문을 먼저 편집국에 넘겨 신문감으로 정리한다.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -7196,6 +7197,1372 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AnswerID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>QuestionID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>SortOrder</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>AnswerText</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>RequiredEvidenceIDs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>IsCorrect</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>EffectGroupID</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ResultText</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>NextType</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>NextID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>QArchivePattern_Correct</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>QArchivePattern</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>과거 기사와 빈민가 목격담은 같은 방식의 실종이 기록에서 반복해 지워졌음을 보여 준다.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>EvOldArticles, EvSlumWitness</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>신문의 삭제와 목격자의 공포가 같은 빈자리를 가리킨다. 실종은 개인의 불운이 아니라 반복된 구조였다.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>QArchivePattern_Erosion</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>QArchivePattern</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>목격자가 떨었으니, 사라진 사람들은 아직 빈민가 골목에서 이름을 부른다.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EvSlumWitness</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>두려운 증언을 유령의 증거로 바꿨다. 반복을 만든 기록의 손길은 다시 어둠 속으로 숨는다.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>QArchivePattern_Credibility</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>QArchivePattern</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>낡은 기사 몇 장만으로 모든 현재 실종이 같은 범인의 짓이라고 쓴다.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>기사만으로는 현재의 실종을 단정할 수 없다. 시간의 간격과 증언의 빈칸을 무시한 기사거리가 된다.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>QCallPattern_Correct</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>QCallPattern</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>쪽지의 지시와 푸른 천의 표식은 사람을 낙원으로 몰아넣은 같은 호출의 흔적이다.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>EvNote, EvBlueCloth</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>글로 남은 지시와 몸에 남는 표식이 겹친다. 호출은 우연한 폐기물이 아니라 사람을 움직이는 명령이었다.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>QCallPattern_Erosion</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>QCallPattern</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>붉은 쪽지는 읽는 사람마다 제 발로 낙원으로 끌려가게 만든다.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EvNote</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>명령의 흔적을 곧장 저주의 힘으로 바꿨다. 누가 사람을 몰았는지 묻는 질문이 사라진다.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QCallPattern_Credibility</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>QCallPattern</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>푸른 천 하나만으로 공장과 낙원이 같은 명령을 썼다고 발표한다.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>표식 하나는 의심의 출발점일 뿐 연결의 증거는 아니다. 서로 다른 장소를 너무 빨리 한 사건으로 묶었다.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QIpangyuCall_Correct</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>QIpangyuCall</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>붉은 쪽지는 낙원 쪽에서 이판규를 직접 불러낸 호출이다.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>EvNote</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>쪽지의 지시가 이판규의 행선지와 맞물린다. 그는 우연히 달아난 것이 아니라 낙원 쪽 호출에 떠밀렸다.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>QIpangyuCall_Erosion</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>QIpangyuCall</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>이판규를 부른 것은 쪽지가 아니라 공장 안에 남은 의식 그 자체다.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>EvRitualNote</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>의식의 기척을 너무 쉽게 의지로 읽었다. 기록보다 공포가 먼저 결론을 밀어 넣는다.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>QIpangyuCall_Credibility</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>QIpangyuCall</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>푸른 천은 이판규가 공장 인부에게 불려갔다는 명찰이다.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>푸른 천만으로는 누가 누구를 불렀는지 증명할 수 없다. 추측이 기록의 빈칸을 대신했다.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness_Correct</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>붉은 쪽지가 남아 있으므로, 이판규의 호출 이야기는 실제 흔적과 맞닿아 있다.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EvNote</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>발작처럼 흘린 말과 쪽지의 호출이 맞물린다. 그의 말은 죄를 피하려 지어낸 헛소리만은 아니다.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness_Erosion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>이판규는 공장에 남은 노래를 들었기에 이미 의식의 편이 되었다.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>EvRitualNote</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>불안한 기척을 곧장 공모의 증거로 바꿨다. 사람의 말이 의식의 소음 속으로 가라앉는다.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness_Credibility</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>푸른 천이 있었으니 이판규의 진술은 전부 사실이다.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>천 조각 하나로 진술 전체를 보증할 수는 없다. 반박은 근거가 아니라 성급한 단정이 되었다.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>QRitualAccident_Correct</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>QRitualAccident</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>의례실 종이의 순서와 몫은 이 일이 준비된 구조였음을 반박한다.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>EvRitualNote</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>종이에 남은 순서와 숫자는 우발적 광신이라는 설명을 무너뜨린다. 누군가가 사람 수까지 세며 의식을 준비했다.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>QRitualAccident_Erosion</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>QRitualAccident</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>가면의 네 눈이 움직였으니 그날의 광기는 저절로 시작됐다.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>EvMask</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>섬뜩한 인상을 원인으로 단정했다. 두려움은 계획을 읽는 대신 스스로 움직이는 물건을 만들어 낸다.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>QRitualAccident_Credibility</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>QRitualAccident</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>옛 기사에 소란이 적혔으니, 그날은 준비 없는 난동이었다.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>기사의 소란이라는 표현만으로 준비 여부를 가를 수 없다. 요약 문장이 현장의 구조를 지웠다.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>QRitualErasure_Correct</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>QRitualErasure</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>악보의 노래와 의례실 기록은 사람의 이름을 흐리고 배역으로 바꾸는 정해진 절차다.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>EvRitualScore, EvRitualNote</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>노래의 결과 기록의 순서가 맞물린다. 의식은 사람을 단번에 없애지 않고, 이름부터 의례의 몫으로 바꿨다.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>QRitualErasure_Erosion</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>QRitualErasure</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>악보를 읽는 순간 노래가 내 이름까지 지워 버린다.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>EvRitualScore</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>eff_question_both</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>의식의 위험을 현재의 확정된 운명으로 발표했다. 공포가 기록을 잠식하며, 남길 문장마저 흔들린다.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>QRitualErasure_Credibility</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>QRitualErasure</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>의례실 종이 한 장만으로 노래가 모든 사람의 이름을 지웠다고 단정한다.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>종이는 절차의 일부를 보여 줄 뿐 노래의 작동 전체를 증명하지 않는다. 한 조각을 결론으로 삼았다.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>QRitualLead_Correct</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>QRitualLead</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>감응 악보와 의례실 기록은 누군가가 순서와 사람 수를 세며 의식을 주도했음을 보여 준다.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>EvRitualScore, EvRitualNote</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>악보의 결과 기록의 숫자가 같은 구조를 가리킨다. 낙원의 의식은 우발적 소문이 아니라 누군가 끝까지 쥔 판이었다.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>QRitualLead_Erosion</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>QRitualLead</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>가면의 눈이 나를 바라보았으니, 가면 자체가 의식을 주도했다.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>EvMask</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>시선의 감각을 주체의 증거로 삼았다. 사람과 물건의 경계가 흐려질수록 기록은 멀어진다.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>QRitualLead_Credibility</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>QRitualLead</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>30</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>낡은 기사에 이름이 없으니 신문사가 의식을 주도했다.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>삭제된 이름은 은폐의 흔적이지 주도자의 서명은 아니다. 빈칸을 범인으로 발표할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose_Correct</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>청색 한복과 네 눈 가면은 4호실이 사람을 의례의 배역으로 준비시키던 곳임을 보여 준다.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>EvBlueHanbok, EvMask</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>의복과 가면은 장식이 아니라 역할을 갈아 끼우는 도구였다. 4호실은 사람을 의례의 몫으로 준비시키던 자리다.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose_Erosion</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>일기에 남은 이름이 흐려졌으니 4호실 벽이 사람의 이름을 먹었다.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>EvDiary</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>사람을 지운 구조를 방의 괴물로 바꿔 버렸다. 벽보다 그 벽을 사용한 이들이 먼저 사라진다.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose_Credibility</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>QRoom4Purpose</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>청색 한복 하나가 있으니 4호실은 단순한 분장실이었다.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>한 벌의 옷만으로 방의 용도를 줄여 버렸다. 가면과 기록이 가리키는 강제의 구조를 놓쳤다.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing_Correct</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>송금은 일기에 적힌 대로 의례의 배역으로 밀려 들어가며 사라졌다.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>EvDiary</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>일기는 송금의 실종이 도피가 아니라, 사람을 의례의 몫으로 바꾸는 순서 안에서 벌어진 소거였음을 남긴다.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing_Erosion</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>20</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>청색 한복이 송금의 몸을 삼켜 낙원 안으로 데려갔다.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>EvBlueHanbok</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>의복에 남은 기척을 사람의 운명으로 덮어썼다. 남은 기록을 읽기보다 공포가 빈자리를 채운다.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing_Credibility</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>30</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>낡은 기사에 실종이 적혔으니 송금도 같은 날 도망쳤다.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>기사의 반복은 구조를 암시할 뿐 송금의 행적을 확정하지 않는다. 시대와 사람을 억지로 한 줄에 묶었다.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway_Correct</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>일기는 송금에게 도망칠 틈이 없었고, 의례의 배역으로 정해졌음을 보여 준다.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>EvDiary</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>송금의 실종은 스스로 떠난 도피가 아니다. 선택당한 사람을 지워 버리는 의례의 순서가 그를 밀어 넣었다.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway_Erosion</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>20</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>송금은 청색 한복을 입는 순간 자기 이름을 버리고 사라지기로 했다.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>EvBlueHanbok</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>eff_question_erosion</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>옷의 상징을 송금의 자발적 선택으로 바꿔 버렸다. 의식이 강요한 자리에 그의 목소리는 남지 않는다.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway_Credibility</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>QSonggeumRunaway</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>옛 기사에도 도망자가 있었으니 송금도 같은 방식으로 달아났다.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>eff_question_credibility</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>과거 기사는 반복을 의심하게 할 뿐, 송금의 선택을 말해 주지 않는다. 비교가 증언을 대신했다.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -7610,7 +8977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7662,7 +9029,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -7768,10 +9135,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>QuestionAnswerTable</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>StateDescriptorTable</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11195,7 +12572,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>scene_ending_erosion</t>
+          <t>scene_gameover_erosion</t>
         </is>
       </c>
     </row>
@@ -11210,7 +12587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11798,7 +13175,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>eff_r9_document</t>
+          <t>eff_question_both</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -11808,7 +13185,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -11818,7 +13195,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>eff_r9_follow_sound</t>
+          <t>eff_question_both</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -11828,37 +13205,37 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>Credibility</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>eff_r9_songsoon_support</t>
+          <t>eff_question_credibility</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TrustChange</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Songsoon</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>1</v>
+          <t>GaugeChange</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>eff_ritual_wrong</t>
+          <t>eff_question_erosion</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -11868,17 +13245,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>eff_room4_conclusion_wrong</t>
+          <t>eff_r9_document</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -11892,13 +13269,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>eff_room4_note_match</t>
+          <t>eff_r9_follow_sound</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -11908,7 +13285,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -11918,47 +13295,47 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>eff_slum_hanbok_press</t>
+          <t>eff_r9_songsoon_support</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GaugeChange</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Erosion</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
+          <t>TrustChange</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Songsoon</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>eff_songsoon_trust</t>
+          <t>eff_ritual_wrong</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TrustChange</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Songsoon</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>1</v>
+          <t>GaugeChange</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>eff_songsoon_wrong</t>
+          <t>eff_room4_conclusion_wrong</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -11978,20 +13355,100 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>eff_room4_note_match</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>GaugeChange</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>eff_slum_hanbok_press</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GaugeChange</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Erosion</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>eff_songsoon_trust</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TrustChange</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Songsoon</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>eff_songsoon_wrong</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GaugeChange</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>eff_threshold_erosion_touch</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>GaugeChange</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Erosion</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12006,7 +13463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12070,6 +13527,16 @@
           <t>InvestigationHint</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ForcedQuestionIDs</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>QuestionMode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -12095,6 +13562,17 @@
           <t>assets/sfx/ambient.mp3</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>첫 기록</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>법정에서 지워진 흔적을 어떤 기록으로 남길지 정한다.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12120,6 +13598,7 @@
           <t>assets/sfx/newsroom.mp3</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12145,6 +13624,7 @@
           <t>assets/sfx/newsroom.mp3</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12190,6 +13670,7 @@
           <t>법정 기록, 누락된 피해 기록, 편집장의 금지선 가운데 두 가지를 확인해 취재의 출발점을 정하세요.</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12215,6 +13696,7 @@
           <t>assets/sfx/newsroom.mp3</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12260,6 +13742,7 @@
           <t>점장의 입, 여급들의 빚, 구석 손님의 침묵 가운데 어디를 먼저 건드릴지 정하세요.</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12285,6 +13768,7 @@
           <t>assets/sfx/creepy.mp3</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12313,6 +13797,16 @@
       <c r="F9" t="n">
         <v>3</v>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>QIpangyuCall</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12338,6 +13832,7 @@
           <t>assets/sfx/tense.mp3</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12366,6 +13861,7 @@
       <c r="F11" t="n">
         <v>1</v>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12394,6 +13890,7 @@
       <c r="F12" t="n">
         <v>1</v>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12422,6 +13919,7 @@
       <c r="F13" t="n">
         <v>3</v>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12457,6 +13955,16 @@
           <t>네가 가진 것이 이 사건과 연결된 증거라는 걸 보여줘야 송순이 입을 연다.</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>QIpangyuMadness, QCallPattern</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12482,6 +13990,7 @@
           <t>assets/sfx/sad.mp3</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12527,6 +14036,7 @@
           <t>벽의 흔적, 남겨진 기록, 송순의 흔들림 가운데 어디부터 잡아야 사건의 구조가 드러나는지 고르세요.</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12562,6 +14072,16 @@
           <t>의식의 계획성과 송금의 실종을 함께 보여 주는 단서를 골라야 한다.</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>QSonggeumMissing, QSonggeumRunaway, QRoom4Purpose</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12587,6 +14107,7 @@
           <t>assets/sfx/mystery.mp3</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12612,6 +14133,7 @@
           <t>assets/sfx/mystery.mp3</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12637,6 +14159,7 @@
           <t>assets/sfx/tense.mp3</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -12662,6 +14185,7 @@
           <t>assets/sfx/mystery.mp3</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12687,6 +14211,7 @@
           <t>assets/sfx/mystery.mp3</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12712,6 +14237,7 @@
           <t>assets/sfx/mystery.mp3</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -12747,6 +14273,7 @@
           <t>그가 직접 연관된 증거를 꺼내야만 그의 입이 열린다. 무관한 것을 내밀면 외면한다.</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12782,6 +14309,7 @@
           <t>자료실 기사 위에 지금 가진 단서를 직접 겹쳐 보며, 무엇이 같은 손에 의해 지워졌는지 확인한다.</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -12827,6 +14355,16 @@
           <t>여자가 파는 믿음, 뒤에 숨은 사내, 최근에 사라진 이들의 흔적 가운데 어디를 먼저 건드릴지 정하세요.</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>QArchivePattern</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -12862,6 +14400,7 @@
           <t>결근·세탁 기록과 출입 동선을 서로 다른 두 축으로 확인해, 사라짐과 지하 문을 연결한다.</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12897,6 +14436,7 @@
           <t>옥련이 알고 있는 것과 연결된 단서만이 그녀의 입을 더 열게 한다.</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -12922,6 +14462,7 @@
           <t>assets/sfx/jazz_dark.mp3</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -12947,6 +14488,7 @@
           <t>assets/sfx/jazz_dark.mp3</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12972,6 +14514,7 @@
           <t>assets/sfx/creepy_2.mp3</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13000,6 +14543,7 @@
       <c r="F32" t="n">
         <v>3</v>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13045,6 +14589,7 @@
           <t>노랫소리, 문 안의 배치, 송순의 호흡 가운데 두 가지를 확인하고 의례실에 들어갈 준비를 하세요.</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13070,6 +14615,7 @@
           <t>assets/sfx/creepy_2.mp3</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -13105,6 +14651,7 @@
           <t>송금이 자발적 무녀가 아니라 강제로 편입됐음을 확인하고, 이번 밤 끊어야 할 순번을 읽는다.</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13133,6 +14680,7 @@
       <c r="F36" t="n">
         <v>1</v>
       </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13171,6 +14719,16 @@
           <t>의례실에서 붙든 구조와 단서를 지금 이 자리의 흔적에 겹쳐, 무엇이 반복되고 있는지 더 분명하게 확인한다.</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>QRitualLead, QRitualAccident, QRitualErasure</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13216,6 +14774,7 @@
           <t>올바른 증거를 고르면 신용이 오른다. 맞지 않는 증거를 내밀면 기사의 신뢰가 흔들린다.</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13241,6 +14800,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13266,6 +14826,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13291,6 +14852,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13316,6 +14878,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -13341,6 +14904,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -13369,6 +14933,7 @@
       <c r="F44" t="n">
         <v>2</v>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -13394,6 +14959,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -13429,6 +14995,7 @@
           <t>폭로로 만든 틈을 어디에 쓸지 고른다. 사람을 붙들거나, 의식을 끊거나, 기록을 남긴다.</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -13457,6 +15024,7 @@
       <c r="F47" t="n">
         <v>2</v>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -13482,6 +15050,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -13507,6 +15076,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -13532,6 +15102,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -13557,6 +15128,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -13595,6 +15167,7 @@
           <t>송금, 이해심, 그리고 이 방에 쌓인 질문들 사이에서 무엇을 사람 쪽으로 남길지 지금 결정한다.</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -13620,6 +15193,7 @@
           <t>assets/sfx/ritual.mp3</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -13645,6 +15219,7 @@
           <t>assets/sfx/ritual_climax.mp3</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -13670,6 +15245,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -13695,6 +15271,7 @@
           <t>assets/sfx/ending.mp3</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: complete forced question checkpoints
</commit_message>
<xml_diff>
--- a/content/generated/script.generated.xlsx
+++ b/content/generated/script.generated.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-12 23:05:24</t>
+          <t>2026-08-12 23:45:27</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CG_QR_IpangyuSeen_01</t>
+          <t>CG_QR_CheckpointFactoryShock</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CG_QR_IpangyuSeen_01</t>
+          <t>CG_QR_CheckpointWell</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -6599,7 +6599,11 @@
           <t>Witness</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CG_QR_CheckpointWell</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>[]</t>
@@ -6667,7 +6671,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_01, CG_QR_SonggeumOpen_02, CG_QR_SonggeumOpen_03, CG_QR_SonggeumOpen_04</t>
+          <t>CG_QR_CheckpointRoom4Conclusion</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -6750,7 +6754,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_01, CG_QR_SonggeumOpen_02, CG_QR_SonggeumOpen_03, CG_QR_SonggeumOpen_04</t>
+          <t>CG_QR_CheckpointRoom4Conclusion</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -6836,7 +6840,11 @@
           <t>Missing</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CG_QR_CheckpointRoom4Conclusion</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>[]</t>
@@ -6904,7 +6912,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CG_QR_RitualOpen_01, CG_QR_RitualOpen_02, CG_QR_RitualOpen_03</t>
+          <t>CG_QR_CheckpointRitualRoom</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -6992,7 +7000,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CG_QR_RitualOpen_01, CG_QR_RitualOpen_02, CG_QR_RitualOpen_03</t>
+          <t>CG_QR_CheckpointRitualRoom</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -7078,7 +7086,11 @@
           <t>Record</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CG_QR_CheckpointSlum</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>[]</t>
@@ -7144,7 +7156,11 @@
           <t>Ritual</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CG_QR_CheckpointRitualRoom</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>[]</t>
@@ -7289,7 +7305,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -7335,7 +7351,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -7377,7 +7393,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -7419,7 +7435,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -7465,7 +7481,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -7507,7 +7523,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -7549,7 +7565,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -7595,7 +7611,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -7637,7 +7653,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -7679,7 +7695,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -7725,7 +7741,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -7767,7 +7783,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -7809,7 +7825,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -7855,7 +7871,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -7897,7 +7913,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -7939,7 +7955,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -7985,7 +8001,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -8027,7 +8043,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -8069,7 +8085,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -8115,7 +8131,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -8157,7 +8173,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -8199,7 +8215,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -8245,7 +8261,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -8287,7 +8303,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -8329,7 +8345,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -8375,7 +8391,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -8417,7 +8433,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -8459,7 +8475,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -8505,7 +8521,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -8547,7 +8563,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Resume</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -8999,7 +9015,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -9163,7 +9179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10859,22 +10875,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cond_RR_QIpangyuSeen_01</t>
+          <t>Cond_QR_CheckpointFactoryShock_01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CG_QR_IpangyuSeen_01</t>
+          <t>CG_QR_CheckpointFactoryShock</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RevealedCharacter</t>
+          <t>SceneVisited</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Ipangyu</t>
+          <t>ch2_factory_shock</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -10891,52 +10907,54 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualOpen_01</t>
+          <t>Cond_QR_CheckpointRitualRoom_01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CG_QR_RitualOpen_01</t>
+          <t>CG_QR_CheckpointRitualRoom</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>SceneVisited</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ReadRitualScore</t>
+          <t>ch5_ritual_room</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>1</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualOpen_02</t>
+          <t>Cond_QR_CheckpointRoom4Conclusion_01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CG_QR_RitualOpen_02</t>
+          <t>CG_QR_CheckpointRoom4Conclusion</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RevealedCharacter</t>
+          <t>SceneVisited</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Haesim</t>
+          <t>ch3_room4_conclusion</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -10953,47 +10971,54 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualOpen_03</t>
+          <t>Cond_QR_CheckpointSlum_01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CG_QR_RitualOpen_03</t>
+          <t>CG_QR_CheckpointSlum</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SceneProgressIndex</t>
+          <t>SceneVisited</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ch4a_slum</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>31</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumOpen_01</t>
+          <t>Cond_QR_CheckpointWell_01</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_01</t>
+          <t>CG_QR_CheckpointWell</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>SceneVisited</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>EvDiary</t>
+          <t>ch2_well</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -11010,22 +11035,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumOpen_02</t>
+          <t>Cond_RR_QIpangyuSeen_01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_02</t>
+          <t>CG_QR_IpangyuSeen_01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>RevealedCharacter</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>EvOldArticles</t>
+          <t>Ipangyu</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -11042,17 +11067,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumOpen_03</t>
+          <t>Cond_RR_QRitualOpen_01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_03</t>
+          <t>CG_QR_RitualOpen_01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SceneProgressIndex</t>
+          <t>GaugeValue</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ReadRitualScore</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -11061,18 +11091,18 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumOpen_04</t>
+          <t>Cond_RR_QRitualOpen_02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CG_QR_SonggeumOpen_04</t>
+          <t>CG_QR_RitualOpen_02</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -11082,7 +11112,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Songgeum</t>
+          <t>Haesim</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -11099,84 +11129,79 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cond_RR_QIpangyuState_00</t>
+          <t>Cond_RR_QRitualOpen_03</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CG_QS_IpangyuCall_01</t>
+          <t>CG_QR_RitualOpen_03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>QuestionSolved_QIpangyuCall</t>
+          <t>SceneProgressIndex</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cond_RR_QIpangyuState_01</t>
+          <t>Cond_RR_QSonggeumOpen_01</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CG_QS_IpangyuCall_02</t>
+          <t>CG_QR_SonggeumOpen_01</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>EvDiary</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>1</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cond_RR_QIpangyuMadnessState_00</t>
+          <t>Cond_RR_QSonggeumOpen_02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CG_QS_IpangyuMadness_01</t>
+          <t>CG_QR_SonggeumOpen_02</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>QuestionSolved_QIpangyuMadness</t>
+          <t>EvOldArticles</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -11193,54 +11218,47 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cond_RR_QIpangyuMadnessState_01</t>
+          <t>Cond_RR_QSonggeumOpen_03</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CG_QS_IpangyuMadness_02</t>
+          <t>CG_QR_SonggeumOpen_03</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>EvNote</t>
+          <t>SceneProgressIndex</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualAccidentState_00</t>
+          <t>Cond_RR_QSonggeumOpen_04</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CG_QS_RitualAccident_01</t>
+          <t>CG_QR_SonggeumOpen_04</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>RevealedCharacter</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>QuestionSolved_QRitualAccident</t>
+          <t>Songgeum</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -11257,22 +11275,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualAccidentState_01</t>
+          <t>Cond_RR_QIpangyuState_00</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CG_QS_RitualAccident_02</t>
+          <t>CG_QS_IpangyuCall_01</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>EvRitualNote</t>
+          <t>QuestionSolved_QIpangyuCall</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -11289,84 +11307,84 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualState_00</t>
+          <t>Cond_RR_QIpangyuState_01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CG_QS_RitualLead_01</t>
+          <t>CG_QS_IpangyuCall_02</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>GaugeValue</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>QuestionSolved_QRitualLead</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cond_RR_QRitualState_01</t>
+          <t>Cond_RR_QIpangyuMadnessState_00</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CG_QS_RitualLead_02</t>
+          <t>CG_QS_IpangyuMadness_01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ReadRitualScore</t>
+          <t>QuestionSolved_QIpangyuMadness</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F70" t="n">
-        <v>1</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumState_00</t>
+          <t>Cond_RR_QIpangyuMadnessState_01</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CG_QS_SonggeumMissing_01</t>
+          <t>CG_QS_IpangyuMadness_02</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>QuestionSolved_QSonggeumMissing</t>
+          <t>EvNote</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -11383,22 +11401,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumState_01</t>
+          <t>Cond_RR_QRitualAccidentState_00</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CG_QS_SonggeumMissing_02</t>
+          <t>CG_QS_RitualAccident_01</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>EvDiary</t>
+          <t>QuestionSolved_QRitualAccident</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -11415,22 +11433,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumRunawayState_00</t>
+          <t>Cond_RR_QRitualAccidentState_01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CG_QS_SonggeumRunaway_01</t>
+          <t>CG_QS_RitualAccident_02</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>QuestionSolved_QSonggeumRunaway</t>
+          <t>EvRitualNote</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -11447,22 +11465,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Cond_RR_QSonggeumRunawayState_01</t>
+          <t>Cond_RR_QRitualState_00</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CG_QS_SonggeumRunaway_02</t>
+          <t>CG_QS_RitualLead_01</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>EvDiary</t>
+          <t>QuestionSolved_QRitualLead</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -11479,44 +11497,42 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Cond_RitualRoom_OldArticles_01</t>
+          <t>Cond_RR_QRitualState_01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>CG_RitualRoom_OldArticles</t>
+          <t>CG_QS_RitualLead_02</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>GaugeValue</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>EvOldArticles</t>
+          <t>ReadRitualScore</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cond_RitualRoom_AccidentSolved_01</t>
+          <t>Cond_RR_QSonggeumState_00</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CG_RitualRoom_QRitualAccident</t>
+          <t>CG_QS_SonggeumMissing_01</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -11526,7 +11542,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>QuestionSolved_QRitualAccident</t>
+          <t>QuestionSolved_QSonggeumMissing</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -11543,22 +11559,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Cond_RitualRoom_QRitualAccident_01</t>
+          <t>Cond_RR_QSonggeumState_01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CG_RitualRoom_QRitualAccident</t>
+          <t>CG_QS_SonggeumMissing_02</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>QuestionSolved</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>QuestionSolved_QRitualAccident</t>
+          <t>EvDiary</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -11575,22 +11591,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cond_RitualRoom_RitualScore_01</t>
+          <t>Cond_RR_QSonggeumRunawayState_00</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CG_RitualRoom_RitualScore</t>
+          <t>CG_QS_SonggeumRunaway_01</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>EvRitualScore</t>
+          <t>QuestionSolved_QSonggeumRunaway</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -11607,102 +11623,108 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Cond_RitualScene_Resonance_01</t>
+          <t>Cond_RR_QSonggeumRunawayState_01</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CG_RitualScene_Resonance2</t>
+          <t>CG_QS_SonggeumRunaway_02</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>EvDiary</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F79" t="n">
-        <v>2</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Cond_RitualScene_SolvedHigh_01</t>
+          <t>Cond_RitualRoom_OldArticles_01</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CG_RitualScene_SolvedHigh</t>
+          <t>CG_RitualRoom_OldArticles</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SolvedQuestionCount</t>
+          <t>EvOldArticles</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F80" t="n">
-        <v>7</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Cond_Ritual_Erosion6_01</t>
+          <t>Cond_RitualRoom_AccidentSolved_01</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CG_Ritual_Erosion6</t>
+          <t>CG_RitualRoom_QRitualAccident</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>QuestionSolved_QRitualAccident</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F81" t="n">
-        <v>6</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Cond_Ritual_QRoom4Purpose_01</t>
+          <t>Cond_RitualRoom_QRitualAccident_01</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CG_Ritual_QRoom4Purpose</t>
+          <t>CG_RitualRoom_QRitualAccident</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -11712,7 +11734,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>QuestionSolved_QRoom4Purpose</t>
+          <t>QuestionSolved_QRitualAccident</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -11729,12 +11751,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Cond_Room4_HasNote_01</t>
+          <t>Cond_RitualRoom_RitualScore_01</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>CG_Room4_HasNote</t>
+          <t>CG_RitualRoom_RitualScore</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -11744,7 +11766,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>EvNote</t>
+          <t>EvRitualScore</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -11761,12 +11783,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Cond_Room4_ReadRitual_01</t>
+          <t>Cond_RitualScene_Resonance_01</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>CG_Room4_ReadRitual</t>
+          <t>CG_RitualScene_Resonance2</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -11776,7 +11798,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ReadRitualScore</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -11785,92 +11807,88 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Cond_Room4_TrustedSongsoon_01</t>
+          <t>Cond_RitualScene_SolvedHigh_01</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>CG_Room4_TrustedSongsoon</t>
+          <t>CG_RitualScene_SolvedHigh</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ChoiceSelected</t>
+          <t>GaugeValue</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Ch3WarehouseTrustSongsoon|Ch3Room4ComfortSongsoon</t>
+          <t>SolvedQuestionCount</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Cond_Slum_HasHanbok_01</t>
+          <t>Cond_Ritual_Erosion6_01</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CG_Slum_HasHanbok</t>
+          <t>CG_Ritual_Erosion6</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>GaugeValue</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>EvBlueHanbok</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Cond_Threshold_CalledEditorFalse_01</t>
+          <t>Cond_Ritual_QRoom4Purpose_01</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>CG_Threshold_CalledEditorFalse</t>
+          <t>CG_Ritual_QRoom4Purpose</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ChoiceSelected</t>
+          <t>QuestionSolved</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Ch5PathNoContact</t>
+          <t>QuestionSolved_QRoom4Purpose</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -11887,42 +11905,44 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Cond_Threshold_Credibility7_01</t>
+          <t>Cond_Room4_HasNote_01</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>CG_Threshold_Credibility7</t>
+          <t>CG_Room4_HasNote</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>EvNote</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F88" t="n">
-        <v>7</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Cond_Threshold_Erosion6_01</t>
+          <t>Cond_Room4_ReadRitual_01</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CG_Threshold_Erosion6</t>
+          <t>CG_Room4_ReadRitual</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -11932,7 +11952,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>ReadRitualScore</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -11941,18 +11961,18 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Cond_Threshold_FoundOldArticles_01</t>
+          <t>Cond_Room4_TrustedSongsoon_01</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>CG_Threshold_FoundOldArticles</t>
+          <t>CG_Room4_TrustedSongsoon</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -11962,7 +11982,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Ch4ALibraryTakeArticles|Ch4ALibraryExposeArchive</t>
+          <t>Ch3WarehouseTrustSongsoon|Ch3Room4ComfortSongsoon</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -11979,104 +11999,106 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Cond_Threshold_Investigation_01</t>
+          <t>Cond_Slum_HasHanbok_01</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CG_Threshold_Investigation3</t>
+          <t>CG_Slum_HasHanbok</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>EvidenceOwned</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Credibility</t>
+          <t>EvBlueHanbok</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F91" t="n">
-        <v>3</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Cond_Threshold_Resonance_01</t>
+          <t>Cond_Threshold_CalledEditorFalse_01</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>CG_Threshold_Resonance2</t>
+          <t>CG_Threshold_CalledEditorFalse</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>GaugeValue</t>
+          <t>ChoiceSelected</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Erosion</t>
+          <t>Ch5PathNoContact</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>GreaterEqual</t>
-        </is>
-      </c>
-      <c r="F92" t="n">
-        <v>2</v>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Cond_Threshold_RitualNote_01</t>
+          <t>Cond_Threshold_Credibility7_01</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CG_Threshold_RitualNote</t>
+          <t>CG_Threshold_Credibility7</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>EvidenceOwned</t>
+          <t>GaugeValue</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>EvRitualNote</t>
+          <t>Credibility</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Cond_Threshold_SolvedMid_01</t>
+          <t>Cond_Threshold_Erosion6_01</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CG_Threshold_SolvedMid</t>
+          <t>CG_Threshold_Erosion6</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -12086,47 +12108,201 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SolvedQuestionCount</t>
+          <t>Erosion</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>[4, 5, 6]</t>
-        </is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>Cond_Threshold_FoundOldArticles_01</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>CG_Threshold_FoundOldArticles</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ChoiceSelected</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Ch4ALibraryTakeArticles|Ch4ALibraryExposeArchive</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Cond_Threshold_Investigation_01</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CG_Threshold_Investigation3</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>GaugeValue</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Cond_Threshold_Resonance_01</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CG_Threshold_Resonance2</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>GaugeValue</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Erosion</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>GreaterEqual</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Cond_Threshold_RitualNote_01</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CG_Threshold_RitualNote</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>EvidenceOwned</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>EvRitualNote</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Cond_Threshold_SolvedMid_01</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CG_Threshold_SolvedMid</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>GaugeValue</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>SolvedQuestionCount</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>[4, 5, 6]</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>Cond_Threshold_TrustedSongsoon_01</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>CG_Threshold_TrustedSongsoon</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>ChoiceSelected</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>Ch3WarehouseTrustSongsoon|Ch3Room4ComfortSongsoon</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>Equal</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>